<commit_message>
refactor: merge upgrade config into skill config
</commit_message>
<xml_diff>
--- a/eoe/Assets/Excels/SkillConfig.xlsx
+++ b/eoe/Assets/Excels/SkillConfig.xlsx
@@ -696,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -707,17 +707,52 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>stat</t>
+          <t>kind</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>heroId</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>heroStat</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>value</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>percent</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>skillId</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>skillStat</t>
         </is>
       </c>
     </row>
@@ -726,12 +761,37 @@
         <v>1001</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="b">
+        <v>3</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -740,13 +800,389 @@
         <v>1002</v>
       </c>
       <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
         <v>10</v>
       </c>
-      <c r="C3" t="n">
+      <c r="H3" t="n">
         <v>0.5</v>
       </c>
-      <c r="D3" t="b">
-        <v>1</v>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>10001</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sharpened Core</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>+1 Attack to all heroes</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>10002</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Vital Plating</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>+4 Max Health to all heroes</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>10003</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Rapid Circuit</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>+0.1 Attack Speed to all heroes</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>30</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>20001</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Edge Calibration</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>+1 Attack</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>20002</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Reinforced Frame</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>+4 Max Health</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>20003</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Critical Lens</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>+5% Crit Chance</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>20004</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tempo Relay</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>+0.1 Attack Speed</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>30001</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Pistol Overclock</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Projectile Speed +2</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1101</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>30002</v>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Pistol Double Tap</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Hit Count +1</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1101</v>
+      </c>
+      <c r="K12" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>